<commit_message>
docs(brief-sheet): add the required Sub Head column to the template
The Content tab of the shipped template had no Sub Head column, but the
form requires a sub head on every content item before submit — so a brief
drafted from the template imported cleanly and then failed validation,
with the planner retyping a sub head for each row by hand.

Adds the column to campaign-brief-template.xlsx (beside Title, with the
sample rows filled so an AI asked to fill the sheet sees the shape) and
to the Content example in CAMPAIGN_BRIEF_SHEET.md. The importer already
reads "Sub Head"/"Subhead" — no code change needed, and sheets without
the column keep importing as before.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/web/templates/campaign-brief-template.xlsx
+++ b/web/templates/campaign-brief-template.xlsx
@@ -702,25 +702,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -731,75 +732,80 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Sub Head</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Platforms</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Asset Sizes</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Publish Date</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Graphic Due Date</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Needs Graphic</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Needs Video</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Caption Direction</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Key Message</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>CTA</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Product Highlight</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Mandatory Text</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Do / Don't</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -813,75 +819,79 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>วากิว A5 ที่กินได้บ่อยกว่าปีละครั้ง</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Photo</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Facebook, Instagram</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>เปิดตัวให้ดูหรู แต่ราคาต้องเด่น</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>วากิว A5 1,290.-</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>จองโต๊ะเลย</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>เนื้อวากิว A5 ลายหินอ่อน</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>ราคารวม VAT แล้ว</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>อย่าใช้ภาพเนื้อสุกเกิน</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -891,59 +901,59 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>เสียงย่างวากิว 5 วิแรก</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Reel</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Instagram, TikTok</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>9:16</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>เสียงย่างเนื้อเป็นพระเอก 5 วิแรก</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>ดูเมนูเต็ม</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -953,66 +963,68 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>เซ็ตวากิว A5 1,290.- ตลอดเดือน ส.ค.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Poster</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>In-store</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>A3 Poster</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>เซ็ตวากิว A5 1,290.-</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>ราคารวม VAT แล้ว</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Asset Sizes: ใส่แค่สัดส่วน (1:1) = ใช้กับทุก platform ในแถว · เจาะจงได้ด้วย 'Instagram: 9:16' คั่นด้วย ; · แถวที่ไม่มี Title จะถูกข้าม</t>
-        </is>
-      </c>
+          <t>Asset Sizes: ใส่แค่สัดส่วน (1:1) = ใช้กับทุก platform ในแถว · เจาะจงได้ด้วย 'Instagram: 9:16' คั่นด้วย ; · แถวที่ไม่มี Title จะถูกข้าม · Title กับ Sub Head ต้องมีทุกแถว</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1166,11 +1178,8 @@
           <t>Central World</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Micro</t>
@@ -1181,7 +1190,6 @@
           <t>TikTok</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>3</t>
@@ -1217,7 +1225,6 @@
           <t>EmQuartier</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>ยังไม่เลือกเพจ</t>
@@ -1351,7 +1358,6 @@
           <t>Other Note</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">

</xml_diff>